<commit_message>
Complete RC10 question scoring, media import and release checks
</commit_message>
<xml_diff>
--- a/public/question-templates/online-week.xlsx
+++ b/public/question-templates/online-week.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Câu hỏi" sheetId="1" r:id="Rb0368abcf4ec4c0f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Thông tin bộ" sheetId="2" r:id="R93c69f9165004cb6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hướng dẫn" sheetId="3" r:id="R068e4c59bef849b9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Câu hỏi" sheetId="1" r:id="Rdb7d8419821647c4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Thông tin bộ" sheetId="2" r:id="Rb70620ccd43041d1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hướng dẫn" sheetId="3" r:id="R2520a65fb9b64acd"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -371,6 +371,8 @@
     <x:col min="29" max="29" width="22" hidden="0" customWidth="1"/>
     <x:col min="30" max="30" width="22" hidden="0" customWidth="1"/>
     <x:col min="31" max="31" width="22" hidden="0" customWidth="1"/>
+    <x:col min="32" max="32" width="64" hidden="0" customWidth="1"/>
+    <x:col min="33" max="33" width="20" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="30" customHeight="1">
@@ -409,6 +411,8 @@
       <x:c r="AC1" s="2"/>
       <x:c r="AD1" s="2"/>
       <x:c r="AE1" s="2"/>
+      <x:c r="AF1" s="2"/>
+      <x:c r="AG1" s="2"/>
     </x:row>
     <x:row r="2" ht="36" customHeight="1">
       <x:c r="A2" s="6" t="str">
@@ -503,6 +507,12 @@
       </x:c>
       <x:c r="AE2" s="6" t="str">
         <x:v>objectiveId</x:v>
+      </x:c>
+      <x:c r="AF2" s="6" t="str">
+        <x:v>allowedGameIds</x:v>
+      </x:c>
+      <x:c r="AG2" s="6" t="str">
+        <x:v>difficulty</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="30" customHeight="1">
@@ -539,6 +549,8 @@
       <x:c r="AC3" s="8" t="str"/>
       <x:c r="AD3" s="8" t="str"/>
       <x:c r="AE3" s="8" t="str"/>
+      <x:c r="AF3" s="8" t="str"/>
+      <x:c r="AG3" s="8" t="str"/>
     </x:row>
     <x:row r="4" ht="30" customHeight="1">
       <x:c r="A4" s="8" t="str"/>
@@ -574,6 +586,8 @@
       <x:c r="AC4" s="8" t="str"/>
       <x:c r="AD4" s="8" t="str"/>
       <x:c r="AE4" s="8" t="str"/>
+      <x:c r="AF4" s="8" t="str"/>
+      <x:c r="AG4" s="8" t="str"/>
     </x:row>
     <x:row r="5" ht="30" customHeight="1">
       <x:c r="A5" s="8" t="str"/>
@@ -609,6 +623,8 @@
       <x:c r="AC5" s="8" t="str"/>
       <x:c r="AD5" s="8" t="str"/>
       <x:c r="AE5" s="8" t="str"/>
+      <x:c r="AF5" s="8" t="str"/>
+      <x:c r="AG5" s="8" t="str"/>
     </x:row>
     <x:row r="6" ht="30" customHeight="1">
       <x:c r="A6" s="8" t="str"/>
@@ -644,6 +660,8 @@
       <x:c r="AC6" s="8" t="str"/>
       <x:c r="AD6" s="8" t="str"/>
       <x:c r="AE6" s="8" t="str"/>
+      <x:c r="AF6" s="8" t="str"/>
+      <x:c r="AG6" s="8" t="str"/>
     </x:row>
     <x:row r="7" ht="30" customHeight="1">
       <x:c r="A7" s="8" t="str"/>
@@ -679,6 +697,8 @@
       <x:c r="AC7" s="8" t="str"/>
       <x:c r="AD7" s="8" t="str"/>
       <x:c r="AE7" s="8" t="str"/>
+      <x:c r="AF7" s="8" t="str"/>
+      <x:c r="AG7" s="8" t="str"/>
     </x:row>
     <x:row r="8" ht="30" customHeight="1">
       <x:c r="A8" s="8" t="str"/>
@@ -714,6 +734,8 @@
       <x:c r="AC8" s="8" t="str"/>
       <x:c r="AD8" s="8" t="str"/>
       <x:c r="AE8" s="8" t="str"/>
+      <x:c r="AF8" s="8" t="str"/>
+      <x:c r="AG8" s="8" t="str"/>
     </x:row>
     <x:row r="9" ht="30" customHeight="1">
       <x:c r="A9" s="8" t="str"/>
@@ -749,6 +771,8 @@
       <x:c r="AC9" s="8" t="str"/>
       <x:c r="AD9" s="8" t="str"/>
       <x:c r="AE9" s="8" t="str"/>
+      <x:c r="AF9" s="8" t="str"/>
+      <x:c r="AG9" s="8" t="str"/>
     </x:row>
     <x:row r="10" ht="30" customHeight="1">
       <x:c r="A10" s="8" t="str"/>
@@ -784,6 +808,8 @@
       <x:c r="AC10" s="8" t="str"/>
       <x:c r="AD10" s="8" t="str"/>
       <x:c r="AE10" s="8" t="str"/>
+      <x:c r="AF10" s="8" t="str"/>
+      <x:c r="AG10" s="8" t="str"/>
     </x:row>
     <x:row r="11" ht="30" customHeight="1">
       <x:c r="A11" s="8" t="str"/>
@@ -819,6 +845,8 @@
       <x:c r="AC11" s="8" t="str"/>
       <x:c r="AD11" s="8" t="str"/>
       <x:c r="AE11" s="8" t="str"/>
+      <x:c r="AF11" s="8" t="str"/>
+      <x:c r="AG11" s="8" t="str"/>
     </x:row>
     <x:row r="12" ht="30" customHeight="1">
       <x:c r="A12" s="8" t="str"/>
@@ -854,6 +882,8 @@
       <x:c r="AC12" s="8" t="str"/>
       <x:c r="AD12" s="8" t="str"/>
       <x:c r="AE12" s="8" t="str"/>
+      <x:c r="AF12" s="8" t="str"/>
+      <x:c r="AG12" s="8" t="str"/>
     </x:row>
     <x:row r="13" ht="30" customHeight="1">
       <x:c r="A13" s="8" t="str"/>
@@ -889,6 +919,8 @@
       <x:c r="AC13" s="8" t="str"/>
       <x:c r="AD13" s="8" t="str"/>
       <x:c r="AE13" s="8" t="str"/>
+      <x:c r="AF13" s="8" t="str"/>
+      <x:c r="AG13" s="8" t="str"/>
     </x:row>
     <x:row r="14" ht="30" customHeight="1">
       <x:c r="A14" s="8" t="str"/>
@@ -924,6 +956,8 @@
       <x:c r="AC14" s="8" t="str"/>
       <x:c r="AD14" s="8" t="str"/>
       <x:c r="AE14" s="8" t="str"/>
+      <x:c r="AF14" s="8" t="str"/>
+      <x:c r="AG14" s="8" t="str"/>
     </x:row>
     <x:row r="15" ht="30" customHeight="1">
       <x:c r="A15" s="8" t="str"/>
@@ -959,6 +993,8 @@
       <x:c r="AC15" s="8" t="str"/>
       <x:c r="AD15" s="8" t="str"/>
       <x:c r="AE15" s="8" t="str"/>
+      <x:c r="AF15" s="8" t="str"/>
+      <x:c r="AG15" s="8" t="str"/>
     </x:row>
     <x:row r="16" ht="30" customHeight="1">
       <x:c r="A16" s="8" t="str"/>
@@ -994,6 +1030,8 @@
       <x:c r="AC16" s="8" t="str"/>
       <x:c r="AD16" s="8" t="str"/>
       <x:c r="AE16" s="8" t="str"/>
+      <x:c r="AF16" s="8" t="str"/>
+      <x:c r="AG16" s="8" t="str"/>
     </x:row>
     <x:row r="17" ht="30" customHeight="1">
       <x:c r="A17" s="8" t="str"/>
@@ -1029,6 +1067,8 @@
       <x:c r="AC17" s="8" t="str"/>
       <x:c r="AD17" s="8" t="str"/>
       <x:c r="AE17" s="8" t="str"/>
+      <x:c r="AF17" s="8" t="str"/>
+      <x:c r="AG17" s="8" t="str"/>
     </x:row>
     <x:row r="18" ht="30" customHeight="1">
       <x:c r="A18" s="8" t="str"/>
@@ -1064,14 +1104,19 @@
       <x:c r="AC18" s="8" t="str"/>
       <x:c r="AD18" s="8" t="str"/>
       <x:c r="AE18" s="8" t="str"/>
+      <x:c r="AF18" s="8" t="str"/>
+      <x:c r="AG18" s="8" t="str"/>
     </x:row>
   </x:sheetData>
-  <x:dataValidations count="2">
+  <x:dataValidations count="3">
     <x:dataValidation type="list" sqref="B3:B902">
       <x:formula1>"quiz,pairs,sentences,numeric-answer,fill-blank,reading-choice,listening-choice,listening-gap"</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="U3:U902">
       <x:formula1>"true,false"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="AG3:AG902">
+      <x:formula1>"easy,medium,hard"</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1150,7 +1195,7 @@
         <x:v>Bộ câu hỏi</x:v>
       </x:c>
       <x:c r="B6" s="15" t="str">
-        <x:v>Mỗi subjectLabel và kind cần 2–30 câu. Một tuần tối đa 30 bộ. Các dòng còn trống được bỏ qua.</x:v>
+        <x:v>Tuần mới có 3–4 môn, tối đa 12 câu/môn qua mọi bộ. Mỗi môn/dạng cần ít nhất 2 câu. Dòng trống được bỏ qua.</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="46" customHeight="1">
@@ -1158,7 +1203,7 @@
         <x:v>Môn và chủ đề</x:v>
       </x:c>
       <x:c r="B7" s="15" t="str">
-        <x:v>subjectLabel, topic, competition, level và week là tên do người soạn tự đặt. Không có danh mục môn bắt buộc.</x:v>
+        <x:v>subjectLabel là tên môn; chọn/xếp môn tại phần xem trước. topic, competition, level và week giữ nhãn tác giả.</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="46" customHeight="1">
@@ -1166,7 +1211,7 @@
         <x:v>Tệp đa phương tiện</x:v>
       </x:c>
       <x:c r="B8" s="15" t="str">
-        <x:v>Tải ảnh PNG/JPEG/WebP và âm thanh MP3/WAV/OGG riêng trong ứng dụng trước khi nhập tài liệu. Điền đúng tên tệp.</x:v>
+        <x:v>Chọn một file Excel cùng ảnh PNG/JPEG/WebP và âm thanh MP3/WAV/OGG trong cùng một lần chọn. Điền đúng tên tệp ở imageFile/audioFile.</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="46" customHeight="1">
@@ -1190,7 +1235,7 @@
         <x:v>Ô nhập</x:v>
       </x:c>
       <x:c r="B11" s="15" t="str">
-        <x:v>Nền vàng nhạt là ô người soạn điền. kind đã điền sẵn để gợi ý dạng câu, không phải câu hỏi mẫu.</x:v>
+        <x:v>Nền vàng nhạt là ô người soạn điền. null (không phân biệt hoa thường) nghĩa là thiếu dữ liệu: cột bắt buộc báo lỗi dòng; cột tùy chọn coi như trống. Lỗi Excel như #NULL! luôn báo lỗi.</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="46" customHeight="1">
@@ -1351,6 +1396,30 @@
       </x:c>
       <x:c r="B32" s="15" t="str">
         <x:v>Nguồn nội dung và quyền sử dụng do người soạn chịu trách nhiệm cung cấp.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="33" ht="46" customHeight="1">
+      <x:c r="A33" s="15" t="str">
+        <x:v>difficulty</x:v>
+      </x:c>
+      <x:c r="B33" s="15" t="str">
+        <x:v>Độ khó từng câu: easy (nền tảng), medium (vận dụng), hard (nâng cao). Gợi ý 4/5/3 trong 12 câu; không chia bộ theo độ khó.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="34" ht="46" customHeight="1">
+      <x:c r="A34" s="15" t="str">
+        <x:v>allowedGameIds</x:v>
+      </x:c>
+      <x:c r="B34" s="15" t="str">
+        <x:v>Tùy chọn giới hạn trò cho từng câu. Để trống dùng mọi trò hỗ trợ. Tách mã bằng |. Ví dụ: memory-match|word-connect.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="35" ht="58" customHeight="1">
+      <x:c r="A35" s="15" t="str">
+        <x:v>Mã trò được nhận</x:v>
+      </x:c>
+      <x:c r="B35" s="15" t="str">
+        <x:v>math-quest, memory-match, sentence-builder, word-connect, sequence-trail. Bộ chỉ mở trò chung cho tất cả câu; giới hạn không ép được trò sai cấu trúc.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>